<commit_message>
Revert spreadsheet instructions to original text
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lab1work.xlsx
+++ b/lab1work.xlsx
@@ -1218,9 +1218,8 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Only update the BLUE portions of the spreadsheet. All pink portions will be automatically updated when you fill in the info for Trial 1, 2, and 3.
-Be sure to also answer the questions about ranking and Big-O.
-Note: Insertion sort only needs times for n = 1,000 through 32,000.</t>
+          <t>Only update the BLUE portions of the spreadsheet. All pink portions will be automatically updated when you fill in the info for Trial 1, 2, and 3. 
+Be sure to also answer the questions about ranking and Big-O</t>
         </is>
       </c>
       <c r="L1" s="9" t="n"/>

</xml_diff>

<commit_message>
Color 'BLUE' text in spreadsheet instructions to match theme blue
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lab1work.xlsx
+++ b/lab1work.xlsx
@@ -1218,8 +1218,20 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Only update the BLUE portions of the spreadsheet. All pink portions will be automatically updated when you fill in the info for Trial 1, 2, and 3. 
+          <r>
+            <t xml:space="preserve">Only update the </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="004472C4"/>
+            </rPr>
+            <t>BLUE</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> portions of the spreadsheet. All pink portions will be automatically updated when you fill in the info for Trial 1, 2, and 3. 
 Be sure to also answer the questions about ranking and Big-O</t>
+          </r>
         </is>
       </c>
       <c r="L1" s="9" t="n"/>

</xml_diff>